<commit_message>
Integrate reviewed enhancement and galaxy baseline while preserving main save policy
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/crew_assignment.xlsx
+++ b/space-battleship/config_excel/crew_assignment.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="crew_assignment" sheetId="1" r:id="Rffd6da574d0e4e38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="crew_assignment" sheetId="1" r:id="Rdaee461206d748b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -665,10 +665,8 @@
       <x:c r="H6" s="7" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I6" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">自动合成背包宝石，并用同类型更高级宝石替换已镶嵌宝石。</x:t>
-        </x:is>
+      <x:c r="I6" s="7" t="str">
+        <x:v>每个配置周期尝试购买1级全局装备强化，正常消耗碎片。</x:v>
       </x:c>
       <x:c r="J6" s="7" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
Upgrade one lowest equipment slot per crew tick
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/crew_assignment.xlsx
+++ b/space-battleship/config_excel/crew_assignment.xlsx
@@ -561,7 +561,7 @@
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>每秒尝试升级全部启用的武器和防御模块，正常消耗资源。</t>
+          <t>每秒按正常费用升级最低等级的一个启用装备槽1级；同级轮流，买不起等待。</t>
         </is>
       </c>
       <c r="J4" s="7" t="inlineStr">
@@ -577,7 +577,7 @@
       <c r="L4" s="7" t="str"/>
       <c r="M4" s="12" t="inlineStr">
         <is>
-          <t>1,10,max</t>
+          <t>1</t>
         </is>
       </c>
     </row>

</xml_diff>